<commit_message>
Sync template styling with Google Sheets
</commit_message>
<xml_diff>
--- a/template dataset MA & NMA.xlsx
+++ b/template dataset MA & NMA.xlsx
@@ -661,12 +661,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
-  <si>
-    <t xml:space="preserve">AUCTUS V2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schema version 2.3</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
+  <si>
+    <t xml:space="preserve">DATASET MA NMA AUCTUS V2.3</t>
   </si>
   <si>
     <t xml:space="preserve">Bagian</t>
@@ -684,37 +681,37 @@
     <t xml:space="preserve">Langkah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Isi satu baris pada analyses untuk setiap analisis yang ingin dijalankan.</t>
+    <t xml:space="preserve">Pada sheet "analyses", isi satu baris untuk setiap satu outcome yang ingin dianalisis.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Isi study_metadata satu kali per study_label untuk seluruh workbook.</t>
+    <t xml:space="preserve">Isi sheet "study_metadata" satu baris per studi. List studi di sheet "study_metadata" berlaku untuk seluruh sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Isi arm_data, effect_data, atau diagnostic_data sesuai sumber data.</t>
+    <t xml:space="preserve">Isi sheet "arm_data", "effect_data", atau "diagnostic_data" sesuai sumber data dan analisis yang direncanakan.</t>
   </si>
   <si>
     <t xml:space="preserve">Kunci outcome</t>
   </si>
   <si>
-    <t xml:space="preserve">outcome_name wajib unik dan menjadi kunci penggabungan analisis. Pilih dari dropdown pada sheet data.</t>
+    <t xml:space="preserve">outcome_name wajib unik dan menjadi kunci penggabungan analisis. outcome_name yang sama = dianalisis menjadi satu hasil.</t>
   </si>
   <si>
     <t xml:space="preserve">Kunci studi</t>
   </si>
   <si>
-    <t xml:space="preserve">study_label wajib unik secara global. Gunakan Smith 2024a, Smith 2024b, atau nama cohort bila diperlukan.</t>
+    <t xml:space="preserve">study_label wajib unik. Gunakan huruf di belakang seperti "Smith 2024a, Smith 2024b", bila ada yang sama nama dan tahunnya.</t>
   </si>
   <si>
     <t xml:space="preserve">Studi multi-arm</t>
   </si>
   <si>
-    <t xml:space="preserve">Masukkan satu baris per arm. Studi 3 arm cukup 3 baris, bukan 3 contrast manual. Tidak perlu ID teknis; arm dikenali dari outcome_name, study_label, dan treatment.</t>
+    <t xml:space="preserve">Di "arm_data", masukkan satu baris per arm/kelompok. Studi 3 arm cukup 3 baris.</t>
   </si>
   <si>
     <t xml:space="preserve">Zero event</t>
@@ -729,12 +726,6 @@
     <t xml:space="preserve">Masukkan OR/RR/HR pada skala natural dan isi CI atau SE.</t>
   </si>
   <si>
-    <t xml:space="preserve">Warna biru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sel input user menggunakan font biru.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Semua baris aktif</t>
   </si>
   <si>
@@ -759,25 +750,19 @@
     <t xml:space="preserve">Sel kuning adalah warning yang harus dibaca sebelum interpretasi.</t>
   </si>
   <si>
-    <t xml:space="preserve">Warna biru muda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sel biru muda adalah informasi tentang keputusan atau eksklusi yang tidak memblokir analisis.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Contoh</t>
   </si>
   <si>
-    <t xml:space="preserve">Lihat CONTOH_PENGISIAN. Sheet read-only tersebut tidak dibaca engine; salin pola ke sheet input.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forest raw</t>
+    <t xml:space="preserve">Lihat CONTOH_PENGISIAN. Sheet read-only tersebut tidak dibaca kode; salin pola ke sheet input.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forest plot raw</t>
   </si>
   <si>
     <t xml:space="preserve">Binary menampilkan Event dan Total per treatment. Continuous menampilkan Mean, SD, dan Total.</t>
   </si>
   <si>
-    <t xml:space="preserve">Forest reported/mixed</t>
+    <t xml:space="preserve">Forest plot reported/mixed</t>
   </si>
   <si>
     <t xml:space="preserve">Forest reported atau mixed hanya menampilkan Total per treatment dan membagi studi menjadi blok Adjusted, Crude, dan Raw-derived. Sample yang tidak dilaporkan tampil sebagai NR.</t>
@@ -789,10 +774,10 @@
     <t xml:space="preserve">Nama treatment pada header dan label Favours dibuat dinamis. lower_better, higher_better, atau neutral harus dipilih berdasarkan arti klinis outcome.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bantuan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jalankan source('meta_nma_engine.R'), lalu hasil &lt;- run_auctus_meta().</t>
+    <t xml:space="preserve">Cara pakai kode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jalankan source('meta_nma_engine.R'), lalu run_auctus_meta().</t>
   </si>
   <si>
     <t xml:space="preserve">CONTOH PENGISIAN, TIDAK DIBACA ENGINE</t>
@@ -1091,11 +1076,28 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF274E13"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <b/>
     </font>
     <font>
       <sz val="18"/>
@@ -1105,23 +1107,12 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <b/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0070C0"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1130,12 +1121,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
+        <fgColor rgb="FF274E13"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -1156,19 +1152,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1187,7 +1192,7 @@
     <tableColumn id="4" name="subgroup_region"/>
     <tableColumn id="5" name="moderator_num_mean_age"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1209,7 +1214,7 @@
     <tableColumn id="12" name="max"/>
     <tableColumn id="13" name="notes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1232,7 +1237,7 @@
     <tableColumn id="13" name="sample2"/>
     <tableColumn id="14" name="notes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1249,17 +1254,17 @@
     <tableColumn id="7" name="threshold"/>
     <tableColumn id="8" name="notes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A4:B24" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="petunjuk" displayName="petunjuk" ref="A4:B22" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
     <tableColumn id="1" name="Bagian"/>
     <tableColumn id="2" name="Penjelasan"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1366,7 +1371,7 @@
     <tableColumn id="8" name="unit"/>
     <tableColumn id="9" name="notes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1650,7 +1655,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF1F4E78"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1664,177 +1669,156 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
+    <row r="4">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" ht="33.75" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" ht="33.75" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" ht="33.75" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" ht="33.75" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" ht="33.75" customHeight="1">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" ht="33.75" customHeight="1">
+      <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="11" ht="33.75" customHeight="1">
+      <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" ht="33.75" customHeight="1">
+      <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="13" ht="33.75" customHeight="1">
+      <c r="A13" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" ht="33.75" customHeight="1">
+      <c r="A14" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="15" ht="33.75" customHeight="1">
+      <c r="A15" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="16" ht="33.75" customHeight="1">
+      <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" ht="33.75" customHeight="1">
+      <c r="A17" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="2" t="s">
+      <c r="B17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="18" ht="33.75" customHeight="1">
+      <c r="A18" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="19" ht="33.75" customHeight="1">
+      <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="2" t="s">
+      <c r="B19" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="20" ht="33.75" customHeight="1">
+      <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B20" t="s">
+    </row>
+    <row r="21" ht="33.75" customHeight="1">
+      <c r="A21" s="3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="2" t="s">
+      <c r="B21" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="22" ht="33.75" customHeight="1">
+      <c r="A22" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="B22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1849,7 +1833,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF70AD47"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1877,899 +1861,899 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="E4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="F4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="G4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="H4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="I4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="3" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="B5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="E5" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="F5" s="8" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="G5" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="H5" s="8"/>
+      <c r="I5" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="B6" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H6" s="8"/>
+      <c r="I6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+      <c r="B7" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4" t="s">
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="4" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="8" t="n">
         <v>64</v>
       </c>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>118</v>
+      </c>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>122</v>
+      </c>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
+      <c r="L40" s="6"/>
+      <c r="M40" s="6"/>
+      <c r="N40" s="6"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="J41" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="M41" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="N41" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G42" s="8" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H42" s="8"/>
+      <c r="I42" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="K42" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="L42" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M42" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="N42" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="6"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4" t="s">
+      <c r="B47" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>188</v>
+      </c>
+      <c r="G47" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C48" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="M25" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>82</v>
-      </c>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
-      <c r="M29" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>122</v>
-      </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>103</v>
-      </c>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>108</v>
-      </c>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4"/>
-      <c r="M36" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="K41" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="M41" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="N41" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4" t="n">
-        <v>95</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="K42" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="L42" s="4" t="n">
-        <v>95</v>
-      </c>
-      <c r="M42" s="4" t="n">
-        <v>96</v>
-      </c>
-      <c r="N42" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C46" s="3" t="s">
+      <c r="D48" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="F48" s="8" t="n">
+        <v>201</v>
+      </c>
+      <c r="G48" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="H48" s="8" t="s">
         <v>129</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>82</v>
-      </c>
-      <c r="D47" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>188</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="H47" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C48" s="4" t="n">
-        <v>74</v>
-      </c>
-      <c r="D48" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E48" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="F48" s="4" t="n">
-        <v>201</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2789,7 +2773,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF1F4E78"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2805,45 +2789,45 @@
     <col min="9" max="9" width="28.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="G1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="H1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="I1" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2888,7 +2872,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2900,29 +2884,29 @@
     <col min="5" max="5" width="25.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>81</v>
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2937,7 +2921,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2957,61 +2941,61 @@
     <col min="13" max="13" width="28.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="I1" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>54</v>
+      <c r="M1" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3044,7 +3028,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -3065,65 +3049,65 @@
     <col min="14" max="14" width="28.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="I1" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="M1" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>54</v>
+      <c r="N1" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3162,7 +3146,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF38761D"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -3177,41 +3161,41 @@
     <col min="8" max="8" width="28.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>54</v>
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3247,80 +3231,80 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>120</v>
+      <c r="E1" s="7" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -3328,10 +3312,10 @@
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>

</xml_diff>